<commit_message>
Update RUN and EQIX models
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EQIX.xlsx
+++ b/EQIX.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dillonwalton/Desktop/business/models/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E267EFC0-1E71-5949-A3D4-0E6904773653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B647F388-5055-4320-9992-E8479AECAC70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="260" yWindow="760" windowWidth="14460" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40020" yWindow="3405" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="Model" sheetId="2" r:id="rId2"/>
+    <sheet name="Data Centers" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -77,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="117">
   <si>
     <t>Q120</t>
   </si>
@@ -383,13 +384,58 @@
   </si>
   <si>
     <t>REIT</t>
+  </si>
+  <si>
+    <t>Enterprise</t>
+  </si>
+  <si>
+    <t>Colocations</t>
+  </si>
+  <si>
+    <t>Company owns building, power and cooling -&gt; customers rent space + bring servers</t>
+  </si>
+  <si>
+    <t>Personal on prem, used internally</t>
+  </si>
+  <si>
+    <t>Hyperscale</t>
+  </si>
+  <si>
+    <t>Managed services / hosted dcs</t>
+  </si>
+  <si>
+    <t>Edge</t>
+  </si>
+  <si>
+    <t>Small facilities to reduce latency</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Reliability</t>
+  </si>
+  <si>
+    <t>Tier I</t>
+  </si>
+  <si>
+    <t>Tier II</t>
+  </si>
+  <si>
+    <t>Tier III</t>
+  </si>
+  <si>
+    <t>Tier IV</t>
+  </si>
+  <si>
+    <t>Mostly through redundancy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -449,6 +495,14 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -458,12 +512,74 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="7">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -472,7 +588,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -482,11 +598,16 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -882,16 +1003,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:I19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="20.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="12">
         <v>35968</v>
       </c>
       <c r="G3" t="s">
@@ -902,10 +1023,10 @@
       </c>
       <c r="I3" s="5">
         <f ca="1">TODAY()</f>
-        <v>46277</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9">
+        <v>46279</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>100</v>
       </c>
@@ -922,7 +1043,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="2:9">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>36</v>
       </c>
@@ -937,7 +1058,7 @@
         <v>102393.58199592</v>
       </c>
     </row>
-    <row r="6" spans="2:9">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>38</v>
       </c>
@@ -955,7 +1076,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:9">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>56</v>
       </c>
@@ -973,7 +1094,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="2:9">
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>58</v>
       </c>
@@ -991,7 +1112,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="2:9">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>41</v>
       </c>
@@ -1002,17 +1123,17 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="2:9">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="2:9">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>43</v>
       </c>
@@ -1023,7 +1144,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="2:5">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>40</v>
       </c>
@@ -1031,7 +1152,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="2:5">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>46</v>
       </c>
@@ -1045,18 +1166,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AV72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.33203125" customWidth="1"/>
+    <col min="24" max="24" width="10.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48">
+    <row r="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:48">
+    <row r="2" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1193,7 +1314,7 @@
         <v>2036</v>
       </c>
     </row>
-    <row r="3" spans="1:48">
+    <row r="3" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1221,7 +1342,7 @@
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
     </row>
-    <row r="4" spans="1:48">
+    <row r="4" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>60</v>
       </c>
@@ -1256,7 +1377,7 @@
         <v>6009</v>
       </c>
     </row>
-    <row r="5" spans="1:48">
+    <row r="5" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>61</v>
       </c>
@@ -1291,7 +1412,7 @@
         <v>4719</v>
       </c>
     </row>
-    <row r="6" spans="1:48">
+    <row r="6" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>62</v>
       </c>
@@ -1326,7 +1447,7 @@
         <v>3203</v>
       </c>
     </row>
-    <row r="7" spans="1:48">
+    <row r="7" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>63</v>
       </c>
@@ -1369,7 +1490,7 @@
         <v>13931</v>
       </c>
     </row>
-    <row r="8" spans="1:48">
+    <row r="8" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1397,7 +1518,7 @@
       <c r="AA8" s="6"/>
       <c r="AB8" s="6"/>
     </row>
-    <row r="9" spans="1:48">
+    <row r="9" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>52</v>
       </c>
@@ -1428,7 +1549,7 @@
       <c r="AA9" s="6"/>
       <c r="AB9" s="6"/>
     </row>
-    <row r="10" spans="1:48">
+    <row r="10" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>51</v>
       </c>
@@ -1459,7 +1580,7 @@
       <c r="AA10" s="6"/>
       <c r="AB10" s="6"/>
     </row>
-    <row r="11" spans="1:48">
+    <row r="11" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>49</v>
       </c>
@@ -1490,7 +1611,7 @@
       <c r="AA11" s="6"/>
       <c r="AB11" s="6"/>
     </row>
-    <row r="12" spans="1:48">
+    <row r="12" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>50</v>
       </c>
@@ -1521,7 +1642,7 @@
       <c r="AA12" s="6"/>
       <c r="AB12" s="6"/>
     </row>
-    <row r="13" spans="1:48">
+    <row r="13" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>48</v>
       </c>
@@ -1552,7 +1673,7 @@
       <c r="AA13" s="6"/>
       <c r="AB13" s="6"/>
     </row>
-    <row r="14" spans="1:48">
+    <row r="14" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -1580,7 +1701,7 @@
       <c r="AA14" s="6"/>
       <c r="AB14" s="6"/>
     </row>
-    <row r="15" spans="1:48">
+    <row r="15" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>94</v>
       </c>
@@ -1611,7 +1732,7 @@
       <c r="AA15" s="6"/>
       <c r="AB15" s="6"/>
     </row>
-    <row r="16" spans="1:48">
+    <row r="16" spans="1:48" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>95</v>
       </c>
@@ -1642,7 +1763,7 @@
       <c r="AA16" s="6"/>
       <c r="AB16" s="6"/>
     </row>
-    <row r="17" spans="2:28">
+    <row r="17" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>96</v>
       </c>
@@ -1673,7 +1794,7 @@
       <c r="AA17" s="6"/>
       <c r="AB17" s="6"/>
     </row>
-    <row r="18" spans="2:28">
+    <row r="18" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>80</v>
       </c>
@@ -1704,7 +1825,7 @@
       <c r="AA18" s="6"/>
       <c r="AB18" s="6"/>
     </row>
-    <row r="19" spans="2:28">
+    <row r="19" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>97</v>
       </c>
@@ -1735,12 +1856,12 @@
       <c r="AA19" s="6"/>
       <c r="AB19" s="6"/>
     </row>
-    <row r="20" spans="2:28">
+    <row r="20" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="2:28">
+    <row r="22" spans="2:28" x14ac:dyDescent="0.25">
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -1768,7 +1889,7 @@
       <c r="AA22" s="6"/>
       <c r="AB22" s="6"/>
     </row>
-    <row r="23" spans="2:28">
+    <row r="23" spans="2:28" x14ac:dyDescent="0.25">
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -1796,7 +1917,7 @@
       <c r="AA23" s="6"/>
       <c r="AB23" s="6"/>
     </row>
-    <row r="24" spans="2:28">
+    <row r="24" spans="2:28" x14ac:dyDescent="0.25">
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -1824,7 +1945,7 @@
       <c r="AA24" s="6"/>
       <c r="AB24" s="6"/>
     </row>
-    <row r="25" spans="2:28">
+    <row r="25" spans="2:28" x14ac:dyDescent="0.25">
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -1852,7 +1973,7 @@
       <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>
     </row>
-    <row r="26" spans="2:28">
+    <row r="26" spans="2:28" x14ac:dyDescent="0.25">
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -1880,7 +2001,7 @@
       <c r="AA26" s="6"/>
       <c r="AB26" s="6"/>
     </row>
-    <row r="27" spans="2:28">
+    <row r="27" spans="2:28" x14ac:dyDescent="0.25">
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -1908,7 +2029,7 @@
       <c r="AA27" s="6"/>
       <c r="AB27" s="6"/>
     </row>
-    <row r="28" spans="2:28">
+    <row r="28" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>64</v>
       </c>
@@ -1945,7 +2066,7 @@
         <v>2377</v>
       </c>
     </row>
-    <row r="29" spans="2:28">
+    <row r="29" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>65</v>
       </c>
@@ -1982,53 +2103,53 @@
         <v>248</v>
       </c>
     </row>
-    <row r="30" spans="2:28">
-      <c r="B30" s="10" t="s">
+    <row r="30" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B30" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="10"/>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="10"/>
-      <c r="X30" s="12">
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="9"/>
+      <c r="O30" s="9"/>
+      <c r="P30" s="9"/>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9"/>
+      <c r="S30" s="9"/>
+      <c r="T30" s="9"/>
+      <c r="U30" s="9"/>
+      <c r="V30" s="9"/>
+      <c r="W30" s="9"/>
+      <c r="X30" s="11">
         <f>SUM(X28:X29)</f>
         <v>2256</v>
       </c>
-      <c r="Y30" s="12">
+      <c r="Y30" s="11">
         <f t="shared" ref="Y30:Z30" si="1">SUM(Y28:Y29)</f>
         <v>0</v>
       </c>
-      <c r="Z30" s="12">
+      <c r="Z30" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AA30" s="12">
+      <c r="AA30" s="11">
         <f>SUM(AA28:AA29)</f>
         <v>2444</v>
       </c>
-      <c r="AB30" s="12">
+      <c r="AB30" s="11">
         <f>SUM(AB28:AB29)</f>
         <v>2625</v>
       </c>
     </row>
-    <row r="31" spans="2:28">
+    <row r="31" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>66</v>
       </c>
@@ -2044,53 +2165,53 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="32" spans="2:28">
-      <c r="B32" s="10" t="s">
+    <row r="32" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B32" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10"/>
-      <c r="L32" s="10"/>
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-      <c r="Q32" s="10"/>
-      <c r="R32" s="10"/>
-      <c r="S32" s="10"/>
-      <c r="T32" s="10"/>
-      <c r="U32" s="10"/>
-      <c r="V32" s="10"/>
-      <c r="W32" s="10"/>
-      <c r="X32" s="12">
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9"/>
+      <c r="O32" s="9"/>
+      <c r="P32" s="9"/>
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9"/>
+      <c r="S32" s="9"/>
+      <c r="T32" s="9"/>
+      <c r="U32" s="9"/>
+      <c r="V32" s="9"/>
+      <c r="W32" s="9"/>
+      <c r="X32" s="11">
         <f>X30-X31</f>
         <v>1172</v>
       </c>
-      <c r="Y32" s="12">
+      <c r="Y32" s="11">
         <f t="shared" ref="Y32:AB32" si="2">Y30-Y31</f>
         <v>0</v>
       </c>
-      <c r="Z32" s="12">
+      <c r="Z32" s="11">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="AA32" s="12">
+      <c r="AA32" s="11">
         <f t="shared" si="2"/>
         <v>1258</v>
       </c>
-      <c r="AB32" s="12">
+      <c r="AB32" s="11">
         <f t="shared" si="2"/>
         <v>1395</v>
       </c>
     </row>
-    <row r="33" spans="2:28">
+    <row r="33" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>69</v>
       </c>
@@ -2106,7 +2227,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="34" spans="2:28">
+    <row r="34" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>68</v>
       </c>
@@ -2122,7 +2243,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="35" spans="2:28">
+    <row r="35" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>70</v>
       </c>
@@ -2138,7 +2259,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="2:28">
+    <row r="36" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>71</v>
       </c>
@@ -2154,7 +2275,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="2:28">
+    <row r="37" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>72</v>
       </c>
@@ -2168,7 +2289,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="2:28">
+    <row r="38" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>77</v>
       </c>
@@ -2182,7 +2303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="2:28">
+    <row r="39" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>73</v>
       </c>
@@ -2207,57 +2328,57 @@
         <v>730</v>
       </c>
     </row>
-    <row r="40" spans="2:28">
-      <c r="B40" s="10" t="s">
+    <row r="40" spans="2:28" x14ac:dyDescent="0.25">
+      <c r="B40" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C40" s="10"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="10"/>
-      <c r="J40" s="10"/>
-      <c r="K40" s="10"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
-      <c r="O40" s="10"/>
-      <c r="P40" s="10"/>
-      <c r="Q40" s="10"/>
-      <c r="R40" s="10"/>
-      <c r="S40" s="10"/>
-      <c r="T40" s="10"/>
-      <c r="U40" s="10"/>
-      <c r="V40" s="10"/>
-      <c r="W40" s="10"/>
-      <c r="X40" s="11">
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="9"/>
+      <c r="L40" s="9"/>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9"/>
+      <c r="O40" s="9"/>
+      <c r="P40" s="9"/>
+      <c r="Q40" s="9"/>
+      <c r="R40" s="9"/>
+      <c r="S40" s="9"/>
+      <c r="T40" s="9"/>
+      <c r="U40" s="9"/>
+      <c r="V40" s="9"/>
+      <c r="W40" s="9"/>
+      <c r="X40" s="10">
         <f>X32-X39</f>
         <v>494</v>
       </c>
-      <c r="Y40" s="11">
+      <c r="Y40" s="10">
         <f t="shared" ref="Y40:AB40" si="4">Y32-Y39</f>
         <v>0</v>
       </c>
-      <c r="Z40" s="11">
+      <c r="Z40" s="10">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="AA40" s="11">
+      <c r="AA40" s="10">
         <f t="shared" si="4"/>
         <v>577</v>
       </c>
-      <c r="AB40" s="11">
+      <c r="AB40" s="10">
         <f t="shared" si="4"/>
         <v>665</v>
       </c>
     </row>
-    <row r="46" spans="2:28">
+    <row r="46" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>75</v>
       </c>
-      <c r="X46" s="9">
+      <c r="X46" s="7">
         <f>X32/X30</f>
         <v>0.51950354609929073</v>
       </c>
@@ -2278,7 +2399,7 @@
         <v>0.53142857142857147</v>
       </c>
     </row>
-    <row r="47" spans="2:28">
+    <row r="47" spans="2:28" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>76</v>
       </c>
@@ -2303,92 +2424,92 @@
         <v>0.25333333333333335</v>
       </c>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>92</v>
       </c>
@@ -2426,4 +2547,105 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId27"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0564E6E4-93FD-411C-99BE-931A48437A94}">
+  <dimension ref="B1:C15"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="C5" s="14"/>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="14"/>
+    </row>
+    <row r="7" spans="2:3" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>112</v>
+      </c>
+      <c r="C11">
+        <v>99.67</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12">
+        <v>99.75</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>114</v>
+      </c>
+      <c r="C13">
+        <v>99.98</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C14">
+        <v>99.995000000000005</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Extend the annual blocks back to each company's first public year
Completes the five data-bearing models: the quarter headers already spanned
each company's public life, and now the annual blocks do too.

  EQIX  +20 years -> 2000..2036
  TSLA  +14 years -> 2010..2030
  RUN   +10 years -> 2015..2035
  BE    already started 2018, its first public year
  GEV   has no annual block

Adds extend_years.ps1, which inserts through Excel for the same reason as the
quarter insert: Excel re-points formulas across the shift where openpyxl would
move cells and leave references behind. It must run after extend_quarters.ps1,
since the annual block sits right of the quarters and moves when they grow.

Verified: formula counts unchanged in all five (158/34/0/72/98), quarter
headers and links untouched, and all 167 workbooks still open in Excel.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EQIX.xlsx
+++ b/EQIX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC54033A-AA55-4924-82CE-F7707955FF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3054D9D-B79E-43A7-BD89-196EDBE41C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1390,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:DW72"/>
+  <dimension ref="A1:EQ72"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
@@ -1398,12 +1398,12 @@
     <col min="103" max="103" width="10.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:147" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:147" x14ac:dyDescent="0.25">
       <c r="C2" s="19" t="s">
         <v>117</v>
       </c>
@@ -1726,58 +1726,118 @@
         <v>28</v>
       </c>
       <c r="DG2">
+        <v>2000</v>
+      </c>
+      <c r="DH2">
+        <v>2001</v>
+      </c>
+      <c r="DI2">
+        <v>2002</v>
+      </c>
+      <c r="DJ2">
+        <v>2003</v>
+      </c>
+      <c r="DK2">
+        <v>2004</v>
+      </c>
+      <c r="DL2">
+        <v>2005</v>
+      </c>
+      <c r="DM2">
+        <v>2006</v>
+      </c>
+      <c r="DN2">
+        <v>2007</v>
+      </c>
+      <c r="DO2">
+        <v>2008</v>
+      </c>
+      <c r="DP2">
+        <v>2009</v>
+      </c>
+      <c r="DQ2">
+        <v>2010</v>
+      </c>
+      <c r="DR2">
+        <v>2011</v>
+      </c>
+      <c r="DS2">
+        <v>2012</v>
+      </c>
+      <c r="DT2">
+        <v>2013</v>
+      </c>
+      <c r="DU2">
+        <v>2014</v>
+      </c>
+      <c r="DV2">
+        <v>2015</v>
+      </c>
+      <c r="DW2">
+        <v>2016</v>
+      </c>
+      <c r="DX2">
+        <v>2017</v>
+      </c>
+      <c r="DY2">
+        <v>2018</v>
+      </c>
+      <c r="DZ2">
+        <v>2019</v>
+      </c>
+      <c r="EA2">
         <v>2020</v>
       </c>
-      <c r="DH2">
+      <c r="EB2">
         <v>2021</v>
       </c>
-      <c r="DI2">
+      <c r="EC2">
         <v>2022</v>
       </c>
-      <c r="DJ2">
+      <c r="ED2">
         <v>2023</v>
       </c>
-      <c r="DK2">
+      <c r="EE2">
         <v>2024</v>
       </c>
-      <c r="DL2">
+      <c r="EF2">
         <v>2025</v>
       </c>
-      <c r="DM2">
+      <c r="EG2">
         <v>2026</v>
       </c>
-      <c r="DN2">
+      <c r="EH2">
         <v>2027</v>
       </c>
-      <c r="DO2">
+      <c r="EI2">
         <v>2028</v>
       </c>
-      <c r="DP2">
+      <c r="EJ2">
         <v>2029</v>
       </c>
-      <c r="DQ2">
+      <c r="EK2">
         <v>2030</v>
       </c>
-      <c r="DR2">
+      <c r="EL2">
         <v>2031</v>
       </c>
-      <c r="DS2">
+      <c r="EM2">
         <v>2032</v>
       </c>
-      <c r="DT2">
+      <c r="EN2">
         <v>2033</v>
       </c>
-      <c r="DU2">
+      <c r="EO2">
         <v>2034</v>
       </c>
-      <c r="DV2">
+      <c r="EP2">
         <v>2035</v>
       </c>
-      <c r="DW2">
+      <c r="EQ2">
         <v>2036</v>
       </c>
     </row>
-    <row r="3" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:147" x14ac:dyDescent="0.25">
       <c r="CD3" s="1"/>
       <c r="CE3" s="1"/>
       <c r="CF3" s="1"/>
@@ -1805,7 +1865,7 @@
       <c r="DB3" s="1"/>
       <c r="DC3" s="1"/>
     </row>
-    <row r="4" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>29</v>
       </c>
@@ -1840,7 +1900,7 @@
         <v>6009</v>
       </c>
     </row>
-    <row r="5" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>30</v>
       </c>
@@ -1875,7 +1935,7 @@
         <v>4719</v>
       </c>
     </row>
-    <row r="6" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>31</v>
       </c>
@@ -1910,7 +1970,7 @@
         <v>3203</v>
       </c>
     </row>
-    <row r="7" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>32</v>
       </c>
@@ -1953,7 +2013,7 @@
         <v>13931</v>
       </c>
     </row>
-    <row r="8" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:147" x14ac:dyDescent="0.25">
       <c r="CD8" s="1"/>
       <c r="CE8" s="1"/>
       <c r="CF8" s="1"/>
@@ -1981,7 +2041,7 @@
       <c r="DB8" s="6"/>
       <c r="DC8" s="6"/>
     </row>
-    <row r="9" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>33</v>
       </c>
@@ -2012,7 +2072,7 @@
       <c r="DB9" s="6"/>
       <c r="DC9" s="6"/>
     </row>
-    <row r="10" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>34</v>
       </c>
@@ -2043,7 +2103,7 @@
       <c r="DB10" s="6"/>
       <c r="DC10" s="6"/>
     </row>
-    <row r="11" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>35</v>
       </c>
@@ -2074,7 +2134,7 @@
       <c r="DB11" s="6"/>
       <c r="DC11" s="6"/>
     </row>
-    <row r="12" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>36</v>
       </c>
@@ -2105,7 +2165,7 @@
       <c r="DB12" s="6"/>
       <c r="DC12" s="6"/>
     </row>
-    <row r="13" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>37</v>
       </c>
@@ -2136,7 +2196,7 @@
       <c r="DB13" s="6"/>
       <c r="DC13" s="6"/>
     </row>
-    <row r="14" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:147" x14ac:dyDescent="0.25">
       <c r="CD14" s="1"/>
       <c r="CE14" s="1"/>
       <c r="CF14" s="1"/>
@@ -2164,7 +2224,7 @@
       <c r="DB14" s="6"/>
       <c r="DC14" s="6"/>
     </row>
-    <row r="15" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>38</v>
       </c>
@@ -2195,7 +2255,7 @@
       <c r="DB15" s="6"/>
       <c r="DC15" s="6"/>
     </row>
-    <row r="16" spans="1:127" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:147" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>39</v>
       </c>

</xml_diff>